<commit_message>
fix(envmon): final-review fixes — empty test-sheet QA gap, batch-miss diagnostics, e2e isolation
Five fixes from the final whole-branch review of slice-2b dialect support:
- equis_reader: gate test-sheet merge on `test_rows or profile.test_sheet`
  so an empty EPAR4_TST_v1 sheet still emits equis_missing_test WARNs
  instead of silently importing every row with empty test-side fields
- remove dead `import pytest` from test_equis_xlsx_engine.py
- equis_missing_batch WARN includes the analysis_date discriminator when
  join_date is True, so a date-driven batch miss is distinguishable
- add "Alternatives considered" to the slice-2b ADR
- fix epar4 fixture so the R9 reanalysis pair differs only by
  analysis_time (not also test_type), so the e2e key-distinctness test
  actually exercises the R9 token instead of being masked by test_type
</commit_message>
<xml_diff>
--- a/tests/fixtures/epar4_edd_fixture.xlsx
+++ b/tests/fixtures/epar4_edd_fixture.xlsx
@@ -759,7 +759,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Reanalysis</t>
+          <t>initial</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Reanalysis</t>
+          <t>initial</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">

</xml_diff>